<commit_message>
data(gold): re-review invalid labels against rules 10-12
</commit_message>
<xml_diff>
--- a/data/gold/gold_to_label.xlsx
+++ b/data/gold/gold_to_label.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ewallet-review-analysis\data\gold\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D9D2686-AB2B-4B52-800C-E7ED8C7156BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2EFDFCD-876A-4F44-9B44-BC1DA9262ADB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1932" uniqueCount="1330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1934" uniqueCount="1330">
   <si>
     <t>gold_id</t>
   </si>
@@ -5661,7 +5661,9 @@
       <c r="B108" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="C108" s="2"/>
+      <c r="C108" s="2" t="s">
+        <v>1326</v>
+      </c>
       <c r="D108" s="2"/>
     </row>
     <row r="109" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -5803,7 +5805,9 @@
       <c r="B120" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="C120" s="2"/>
+      <c r="C120" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D120" s="2"/>
     </row>
     <row r="121" spans="1:4" ht="30" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data(gold): fix remaining invalid labels, label reserve rows, rules 13-14
</commit_message>
<xml_diff>
--- a/data/gold/gold_to_label.xlsx
+++ b/data/gold/gold_to_label.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ewallet-review-analysis\data\gold\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38DF155D-30DF-44A0-A75D-7FCC44840EA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBBA17B6-E278-4D70-A86F-A1F85AB2F969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="gold" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1934" uniqueCount="1330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1989" uniqueCount="1331">
   <si>
     <t>gold_id</t>
   </si>
@@ -4011,6 +4011,9 @@
   </si>
   <si>
     <t>sarcasm</t>
+  </si>
+  <si>
+    <t>unsure</t>
   </si>
 </sst>
 </file>
@@ -5206,7 +5209,7 @@
         <v>141</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>1324</v>
+        <v>1326</v>
       </c>
       <c r="D70" s="2"/>
     </row>
@@ -5446,7 +5449,7 @@
         <v>181</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>1324</v>
+        <v>1327</v>
       </c>
       <c r="D90" s="2"/>
     </row>
@@ -5914,7 +5917,7 @@
         <v>259</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>1324</v>
+        <v>1327</v>
       </c>
       <c r="D129" s="2"/>
     </row>
@@ -6324,7 +6327,7 @@
         <v>327</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>1324</v>
+        <v>1327</v>
       </c>
       <c r="D163" s="2"/>
     </row>
@@ -6420,9 +6423,11 @@
         <v>343</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>1324</v>
-      </c>
-      <c r="D171" s="2"/>
+        <v>1326</v>
+      </c>
+      <c r="D171" s="2" t="s">
+        <v>1330</v>
+      </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
@@ -6480,9 +6485,11 @@
         <v>353</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>1324</v>
-      </c>
-      <c r="D176" s="2"/>
+        <v>1327</v>
+      </c>
+      <c r="D176" s="2" t="s">
+        <v>1330</v>
+      </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
@@ -6720,7 +6727,7 @@
         <v>393</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>1324</v>
+        <v>1327</v>
       </c>
       <c r="D196" s="2"/>
     </row>
@@ -6864,7 +6871,7 @@
         <v>417</v>
       </c>
       <c r="C208" s="2" t="s">
-        <v>1324</v>
+        <v>1327</v>
       </c>
       <c r="D208" s="2"/>
     </row>
@@ -8090,7 +8097,7 @@
         <v>621</v>
       </c>
       <c r="C310" s="2" t="s">
-        <v>1324</v>
+        <v>1327</v>
       </c>
       <c r="D310" s="2"/>
     </row>
@@ -9362,7 +9369,7 @@
         <v>833</v>
       </c>
       <c r="C416" s="2" t="s">
-        <v>1324</v>
+        <v>1327</v>
       </c>
       <c r="D416" s="2"/>
     </row>
@@ -9902,7 +9909,7 @@
         <v>923</v>
       </c>
       <c r="C461" s="2" t="s">
-        <v>1326</v>
+        <v>1327</v>
       </c>
       <c r="D461" s="2"/>
     </row>
@@ -10154,9 +10161,11 @@
         <v>965</v>
       </c>
       <c r="C482" s="2" t="s">
-        <v>1324</v>
-      </c>
-      <c r="D482" s="2"/>
+        <v>1325</v>
+      </c>
+      <c r="D482" s="2" t="s">
+        <v>1330</v>
+      </c>
     </row>
     <row r="483" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A483" s="2" t="s">
@@ -10998,9 +11007,11 @@
         <v>1105</v>
       </c>
       <c r="C552" s="2" t="s">
-        <v>1324</v>
-      </c>
-      <c r="D552" s="2"/>
+        <v>1326</v>
+      </c>
+      <c r="D552" s="2" t="s">
+        <v>1330</v>
+      </c>
     </row>
     <row r="553" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A553" s="2" t="s">
@@ -11274,7 +11285,7 @@
         <v>1151</v>
       </c>
       <c r="C575" s="2" t="s">
-        <v>1324</v>
+        <v>1326</v>
       </c>
       <c r="D575" s="2"/>
     </row>
@@ -11737,7 +11748,9 @@
       <c r="B12" s="2" t="s">
         <v>1225</v>
       </c>
-      <c r="C12" s="2"/>
+      <c r="C12" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D12" s="2"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -11747,7 +11760,9 @@
       <c r="B13" s="2" t="s">
         <v>1227</v>
       </c>
-      <c r="C13" s="2"/>
+      <c r="C13" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D13" s="2"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -11757,7 +11772,9 @@
       <c r="B14" s="2" t="s">
         <v>1229</v>
       </c>
-      <c r="C14" s="2"/>
+      <c r="C14" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D14" s="2"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -11767,7 +11784,9 @@
       <c r="B15" s="2" t="s">
         <v>1231</v>
       </c>
-      <c r="C15" s="2"/>
+      <c r="C15" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D15" s="2"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -11777,7 +11796,9 @@
       <c r="B16" s="2" t="s">
         <v>1233</v>
       </c>
-      <c r="C16" s="2"/>
+      <c r="C16" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D16" s="2"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -11787,7 +11808,9 @@
       <c r="B17" s="2" t="s">
         <v>1235</v>
       </c>
-      <c r="C17" s="2"/>
+      <c r="C17" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D17" s="2"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -11797,7 +11820,9 @@
       <c r="B18" s="2" t="s">
         <v>1237</v>
       </c>
-      <c r="C18" s="2"/>
+      <c r="C18" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D18" s="2"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -11807,7 +11832,9 @@
       <c r="B19" s="2" t="s">
         <v>1239</v>
       </c>
-      <c r="C19" s="2"/>
+      <c r="C19" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D19" s="2"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -11817,7 +11844,9 @@
       <c r="B20" s="2" t="s">
         <v>1241</v>
       </c>
-      <c r="C20" s="2"/>
+      <c r="C20" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D20" s="2"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -11827,7 +11856,9 @@
       <c r="B21" s="2" t="s">
         <v>1243</v>
       </c>
-      <c r="C21" s="2"/>
+      <c r="C21" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D21" s="2"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -11837,7 +11868,9 @@
       <c r="B22" s="2" t="s">
         <v>1245</v>
       </c>
-      <c r="C22" s="2"/>
+      <c r="C22" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D22" s="2"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -11847,7 +11880,9 @@
       <c r="B23" s="2" t="s">
         <v>1247</v>
       </c>
-      <c r="C23" s="2"/>
+      <c r="C23" s="2" t="s">
+        <v>1326</v>
+      </c>
       <c r="D23" s="2"/>
     </row>
     <row r="24" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -11857,7 +11892,9 @@
       <c r="B24" s="2" t="s">
         <v>1249</v>
       </c>
-      <c r="C24" s="2"/>
+      <c r="C24" s="2" t="s">
+        <v>1327</v>
+      </c>
       <c r="D24" s="2"/>
     </row>
     <row r="25" spans="1:4" ht="60" x14ac:dyDescent="0.25">
@@ -11867,7 +11904,9 @@
       <c r="B25" s="2" t="s">
         <v>1251</v>
       </c>
-      <c r="C25" s="2"/>
+      <c r="C25" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D25" s="2"/>
     </row>
     <row r="26" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -11877,7 +11916,9 @@
       <c r="B26" s="2" t="s">
         <v>1253</v>
       </c>
-      <c r="C26" s="2"/>
+      <c r="C26" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D26" s="2"/>
     </row>
     <row r="27" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -11887,7 +11928,9 @@
       <c r="B27" s="2" t="s">
         <v>1255</v>
       </c>
-      <c r="C27" s="2"/>
+      <c r="C27" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D27" s="2"/>
     </row>
     <row r="28" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -11897,7 +11940,9 @@
       <c r="B28" s="2" t="s">
         <v>1257</v>
       </c>
-      <c r="C28" s="2"/>
+      <c r="C28" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D28" s="2"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -11907,7 +11952,9 @@
       <c r="B29" s="2" t="s">
         <v>1259</v>
       </c>
-      <c r="C29" s="2"/>
+      <c r="C29" s="2" t="s">
+        <v>1326</v>
+      </c>
       <c r="D29" s="2"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -11917,7 +11964,9 @@
       <c r="B30" s="2" t="s">
         <v>1261</v>
       </c>
-      <c r="C30" s="2"/>
+      <c r="C30" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D30" s="2"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -11927,7 +11976,9 @@
       <c r="B31" s="2" t="s">
         <v>1263</v>
       </c>
-      <c r="C31" s="2"/>
+      <c r="C31" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D31" s="2"/>
     </row>
     <row r="32" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -11937,7 +11988,9 @@
       <c r="B32" s="2" t="s">
         <v>1265</v>
       </c>
-      <c r="C32" s="2"/>
+      <c r="C32" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D32" s="2"/>
     </row>
     <row r="33" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -11947,7 +12000,9 @@
       <c r="B33" s="2" t="s">
         <v>1267</v>
       </c>
-      <c r="C33" s="2"/>
+      <c r="C33" s="2" t="s">
+        <v>1327</v>
+      </c>
       <c r="D33" s="2"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -11957,7 +12012,9 @@
       <c r="B34" s="2" t="s">
         <v>1269</v>
       </c>
-      <c r="C34" s="2"/>
+      <c r="C34" s="2" t="s">
+        <v>1326</v>
+      </c>
       <c r="D34" s="2"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -11967,7 +12024,9 @@
       <c r="B35" s="2" t="s">
         <v>1271</v>
       </c>
-      <c r="C35" s="2"/>
+      <c r="C35" s="2" t="s">
+        <v>1326</v>
+      </c>
       <c r="D35" s="2"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -11977,7 +12036,9 @@
       <c r="B36" s="2" t="s">
         <v>1273</v>
       </c>
-      <c r="C36" s="2"/>
+      <c r="C36" s="2" t="s">
+        <v>1326</v>
+      </c>
       <c r="D36" s="2"/>
     </row>
     <row r="37" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -11987,7 +12048,9 @@
       <c r="B37" s="2" t="s">
         <v>1275</v>
       </c>
-      <c r="C37" s="2"/>
+      <c r="C37" s="2" t="s">
+        <v>1327</v>
+      </c>
       <c r="D37" s="2"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -11997,7 +12060,9 @@
       <c r="B38" s="2" t="s">
         <v>1277</v>
       </c>
-      <c r="C38" s="2"/>
+      <c r="C38" s="2" t="s">
+        <v>1327</v>
+      </c>
       <c r="D38" s="2"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -12007,7 +12072,9 @@
       <c r="B39" s="2" t="s">
         <v>1279</v>
       </c>
-      <c r="C39" s="2"/>
+      <c r="C39" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D39" s="2"/>
     </row>
     <row r="40" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -12017,7 +12084,9 @@
       <c r="B40" s="2" t="s">
         <v>1281</v>
       </c>
-      <c r="C40" s="2"/>
+      <c r="C40" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D40" s="2"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -12027,7 +12096,9 @@
       <c r="B41" s="2" t="s">
         <v>1283</v>
       </c>
-      <c r="C41" s="2"/>
+      <c r="C41" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D41" s="2"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -12037,7 +12108,9 @@
       <c r="B42" s="2" t="s">
         <v>1285</v>
       </c>
-      <c r="C42" s="2"/>
+      <c r="C42" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D42" s="2"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -12047,7 +12120,9 @@
       <c r="B43" s="2" t="s">
         <v>1287</v>
       </c>
-      <c r="C43" s="2"/>
+      <c r="C43" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D43" s="2"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -12057,7 +12132,9 @@
       <c r="B44" s="2" t="s">
         <v>1289</v>
       </c>
-      <c r="C44" s="2"/>
+      <c r="C44" s="2" t="s">
+        <v>1324</v>
+      </c>
       <c r="D44" s="2"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -12067,7 +12144,9 @@
       <c r="B45" s="2" t="s">
         <v>1291</v>
       </c>
-      <c r="C45" s="2"/>
+      <c r="C45" s="2" t="s">
+        <v>1326</v>
+      </c>
       <c r="D45" s="2"/>
     </row>
     <row r="46" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -12077,7 +12156,9 @@
       <c r="B46" s="2" t="s">
         <v>1293</v>
       </c>
-      <c r="C46" s="2"/>
+      <c r="C46" s="2" t="s">
+        <v>1326</v>
+      </c>
       <c r="D46" s="2"/>
     </row>
     <row r="47" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -12087,7 +12168,9 @@
       <c r="B47" s="2" t="s">
         <v>1295</v>
       </c>
-      <c r="C47" s="2"/>
+      <c r="C47" s="2" t="s">
+        <v>1327</v>
+      </c>
       <c r="D47" s="2"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -12097,7 +12180,9 @@
       <c r="B48" s="2" t="s">
         <v>1297</v>
       </c>
-      <c r="C48" s="2"/>
+      <c r="C48" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D48" s="2"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -12107,7 +12192,9 @@
       <c r="B49" s="2" t="s">
         <v>1299</v>
       </c>
-      <c r="C49" s="2"/>
+      <c r="C49" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D49" s="2"/>
     </row>
     <row r="50" spans="1:4" ht="90" x14ac:dyDescent="0.25">
@@ -12117,7 +12204,9 @@
       <c r="B50" s="2" t="s">
         <v>1301</v>
       </c>
-      <c r="C50" s="2"/>
+      <c r="C50" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D50" s="2"/>
     </row>
     <row r="51" spans="1:4" ht="75" x14ac:dyDescent="0.25">
@@ -12127,7 +12216,9 @@
       <c r="B51" s="2" t="s">
         <v>1303</v>
       </c>
-      <c r="C51" s="2"/>
+      <c r="C51" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D51" s="2"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -12137,7 +12228,9 @@
       <c r="B52" s="2" t="s">
         <v>1305</v>
       </c>
-      <c r="C52" s="2"/>
+      <c r="C52" s="2" t="s">
+        <v>1327</v>
+      </c>
       <c r="D52" s="2"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -12147,8 +12240,12 @@
       <c r="B53" s="2" t="s">
         <v>1307</v>
       </c>
-      <c r="C53" s="2"/>
-      <c r="D53" s="2"/>
+      <c r="C53" s="2" t="s">
+        <v>1325</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>1329</v>
+      </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
@@ -12157,7 +12254,9 @@
       <c r="B54" s="2" t="s">
         <v>1309</v>
       </c>
-      <c r="C54" s="2"/>
+      <c r="C54" s="2" t="s">
+        <v>1326</v>
+      </c>
       <c r="D54" s="2"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -12167,7 +12266,9 @@
       <c r="B55" s="2" t="s">
         <v>1311</v>
       </c>
-      <c r="C55" s="2"/>
+      <c r="C55" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D55" s="2"/>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -12177,7 +12278,9 @@
       <c r="B56" s="2" t="s">
         <v>1313</v>
       </c>
-      <c r="C56" s="2"/>
+      <c r="C56" s="2" t="s">
+        <v>1327</v>
+      </c>
       <c r="D56" s="2"/>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -12187,7 +12290,9 @@
       <c r="B57" s="2" t="s">
         <v>1315</v>
       </c>
-      <c r="C57" s="2"/>
+      <c r="C57" s="2" t="s">
+        <v>1324</v>
+      </c>
       <c r="D57" s="2"/>
     </row>
     <row r="58" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -12197,7 +12302,9 @@
       <c r="B58" s="2" t="s">
         <v>1317</v>
       </c>
-      <c r="C58" s="2"/>
+      <c r="C58" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D58" s="2"/>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -12207,7 +12314,9 @@
       <c r="B59" s="2" t="s">
         <v>1319</v>
       </c>
-      <c r="C59" s="2"/>
+      <c r="C59" s="2" t="s">
+        <v>1326</v>
+      </c>
       <c r="D59" s="2"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -12217,7 +12326,9 @@
       <c r="B60" s="2" t="s">
         <v>1321</v>
       </c>
-      <c r="C60" s="2"/>
+      <c r="C60" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D60" s="2"/>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -12227,7 +12338,9 @@
       <c r="B61" s="2" t="s">
         <v>1323</v>
       </c>
-      <c r="C61" s="2"/>
+      <c r="C61" s="2" t="s">
+        <v>1326</v>
+      </c>
       <c r="D61" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data(gold): label final reserve rows R0002-R0008
</commit_message>
<xml_diff>
--- a/data/gold/gold_to_label.xlsx
+++ b/data/gold/gold_to_label.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ewallet-review-analysis\data\gold\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBBA17B6-E278-4D70-A86F-A1F85AB2F969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A046638-A74A-467C-B49A-4E8094311BCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1989" uniqueCount="1331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2000" uniqueCount="1331">
   <si>
     <t>gold_id</t>
   </si>
@@ -11648,7 +11648,9 @@
       <c r="B2" s="2" t="s">
         <v>1205</v>
       </c>
-      <c r="C2" s="2"/>
+      <c r="C2" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D2" s="2"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -11658,7 +11660,9 @@
       <c r="B3" s="2" t="s">
         <v>1207</v>
       </c>
-      <c r="C3" s="2"/>
+      <c r="C3" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D3" s="2"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -11668,7 +11672,9 @@
       <c r="B4" s="2" t="s">
         <v>1209</v>
       </c>
-      <c r="C4" s="2"/>
+      <c r="C4" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -11678,7 +11684,9 @@
       <c r="B5" s="2" t="s">
         <v>1211</v>
       </c>
-      <c r="C5" s="2"/>
+      <c r="C5" s="2" t="s">
+        <v>1326</v>
+      </c>
       <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -11688,7 +11696,9 @@
       <c r="B6" s="2" t="s">
         <v>1213</v>
       </c>
-      <c r="C6" s="2"/>
+      <c r="C6" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -11698,7 +11708,9 @@
       <c r="B7" s="2" t="s">
         <v>1215</v>
       </c>
-      <c r="C7" s="2"/>
+      <c r="C7" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D7" s="2"/>
     </row>
     <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -11708,7 +11720,9 @@
       <c r="B8" s="2" t="s">
         <v>1217</v>
       </c>
-      <c r="C8" s="2"/>
+      <c r="C8" s="2" t="s">
+        <v>1325</v>
+      </c>
       <c r="D8" s="2"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -11718,7 +11732,9 @@
       <c r="B9" s="2" t="s">
         <v>1219</v>
       </c>
-      <c r="C9" s="2"/>
+      <c r="C9" s="2" t="s">
+        <v>1327</v>
+      </c>
       <c r="D9" s="2"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -11728,8 +11744,12 @@
       <c r="B10" s="2" t="s">
         <v>1221</v>
       </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
+      <c r="C10" s="2" t="s">
+        <v>1327</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>1328</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
@@ -11738,7 +11758,9 @@
       <c r="B11" s="2" t="s">
         <v>1223</v>
       </c>
-      <c r="C11" s="2"/>
+      <c r="C11" s="2" t="s">
+        <v>1326</v>
+      </c>
       <c r="D11" s="2"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>